<commit_message>
change fields in the file of customer.xls
</commit_message>
<xml_diff>
--- a/static/Archived/Customers.xlsx
+++ b/static/Archived/Customers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marketingcordinator/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berse\OneDrive\Documents\GitHub\VisualPos\static\Archived\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7E12035-3C5A-9744-8D59-C4766B684C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D7A134-6DEC-4E7D-9E39-735F4C63BCE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>ID</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Cedula</t>
   </si>
@@ -35,6 +32,27 @@
   </si>
   <si>
     <t>Telefono</t>
+  </si>
+  <si>
+    <t>Barrio</t>
+  </si>
+  <si>
+    <t>Direccion</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Ingreso mensual</t>
+  </si>
+  <si>
+    <t>Fuente de ingreso</t>
+  </si>
+  <si>
+    <t>Situacion laboral</t>
+  </si>
+  <si>
+    <t>Producto solicitado</t>
   </si>
 </sst>
 </file>
@@ -50,10 +68,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -64,7 +82,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -74,16 +92,31 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF356854"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF356854"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF284E3F"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF356854"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF284E3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF284E3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF284E3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -91,10 +124,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -398,31 +440,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="13.1640625" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" customWidth="1"/>
-    <col min="4" max="4" width="14.5" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="1" max="5" width="22.5703125" customWidth="1"/>
+    <col min="6" max="6" width="20.85546875" customWidth="1"/>
+    <col min="7" max="7" width="24.85546875" customWidth="1"/>
+    <col min="8" max="8" width="21.85546875" customWidth="1"/>
+    <col min="9" max="9" width="23" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" customWidth="1"/>
+    <col min="11" max="11" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>